<commit_message>
Updating raw data - BORIS additions; BBC, COCO, and 2PP now fully complete and not expecting any new video additions
</commit_message>
<xml_diff>
--- a/raw_data/age_sex_named_subjects.xlsx
+++ b/raw_data/age_sex_named_subjects.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8099077b681ff7d8/Documents/A - UniKonstanz/Thesis/Capuchin_HC_foraging_efficiency_and_selectivity/raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="123" documentId="8_{56112C07-952E-46B1-817F-A8EEFE27D34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3141CE1B-92DE-4226-B3BC-E0332960EA02}"/>
+  <xr:revisionPtr revIDLastSave="142" documentId="8_{56112C07-952E-46B1-817F-A8EEFE27D34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BE47611-F006-4AEB-8168-FAF4004156CA}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{4D44F5B2-B406-4CE5-BE6B-7416F5D6CCF7}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="83">
   <si>
     <t>T</t>
   </si>
@@ -257,9 +257,6 @@
     <t xml:space="preserve">Still need ID matched </t>
   </si>
   <si>
-    <t>Maybe</t>
-  </si>
-  <si>
     <t>age</t>
   </si>
   <si>
@@ -284,13 +281,13 @@
     <t>JUV; Named individual from BBC Stream</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>male</t>
   </si>
   <si>
     <t>female</t>
+  </si>
+  <si>
+    <t>Beanie</t>
   </si>
 </sst>
 </file>
@@ -343,11 +340,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -366,10 +362,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -689,7 +681,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7191118-2807-40F8-9DE6-19E177A1BEC5}">
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14.26953125" customWidth="1"/>
@@ -711,10 +703,10 @@
         <v>58</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>74</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>59</v>
@@ -737,10 +729,10 @@
         <v>61</v>
       </c>
       <c r="E2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G2" t="s">
         <v>3</v>
@@ -763,10 +755,10 @@
         <v>61</v>
       </c>
       <c r="E3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G3" t="s">
         <v>3</v>
@@ -789,10 +781,10 @@
         <v>62</v>
       </c>
       <c r="E4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G4" t="s">
         <v>3</v>
@@ -815,10 +807,10 @@
         <v>63</v>
       </c>
       <c r="E5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G5" t="s">
         <v>3</v>
@@ -841,10 +833,10 @@
         <v>61</v>
       </c>
       <c r="E6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G6" t="s">
         <v>3</v>
@@ -867,10 +859,10 @@
         <v>61</v>
       </c>
       <c r="E7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G7" t="s">
         <v>3</v>
@@ -893,10 +885,10 @@
         <v>61</v>
       </c>
       <c r="E8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G8" t="s">
         <v>3</v>
@@ -919,10 +911,10 @@
         <v>62</v>
       </c>
       <c r="E9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G9" t="s">
         <v>3</v>
@@ -945,10 +937,10 @@
         <v>63</v>
       </c>
       <c r="E10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G10" t="s">
         <v>3</v>
@@ -971,10 +963,10 @@
         <v>64</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F11" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G11" t="s">
         <v>3</v>
@@ -997,10 +989,10 @@
         <v>63</v>
       </c>
       <c r="E12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F12" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G12" t="s">
         <v>3</v>
@@ -1023,10 +1015,10 @@
         <v>61</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F13" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G13" t="s">
         <v>3</v>
@@ -1049,10 +1041,10 @@
         <v>65</v>
       </c>
       <c r="E14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F14" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G14" t="s">
         <v>3</v>
@@ -1075,10 +1067,10 @@
         <v>66</v>
       </c>
       <c r="E15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F15" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G15" t="s">
         <v>3</v>
@@ -1101,10 +1093,10 @@
         <v>64</v>
       </c>
       <c r="E16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F16" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G16" t="s">
         <v>3</v>
@@ -1127,10 +1119,10 @@
         <v>64</v>
       </c>
       <c r="E17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F17" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G17" t="s">
         <v>3</v>
@@ -1153,10 +1145,10 @@
         <v>64</v>
       </c>
       <c r="E18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F18" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G18" t="s">
         <v>3</v>
@@ -1179,10 +1171,10 @@
         <v>64</v>
       </c>
       <c r="E19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G19" t="s">
         <v>3</v>
@@ -1205,10 +1197,10 @@
         <v>64</v>
       </c>
       <c r="E20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F20" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G20" t="s">
         <v>3</v>
@@ -1231,10 +1223,10 @@
         <v>64</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>3</v>
@@ -1256,11 +1248,11 @@
       <c r="D22" t="s">
         <v>61</v>
       </c>
-      <c r="E22" s="3" t="s">
-        <v>75</v>
+      <c r="E22" t="s">
+        <v>74</v>
       </c>
       <c r="F22" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G22" t="s">
         <v>3</v>
@@ -1283,10 +1275,10 @@
         <v>62</v>
       </c>
       <c r="E23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F23" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G23" t="s">
         <v>3</v>
@@ -1309,10 +1301,10 @@
         <v>66</v>
       </c>
       <c r="E24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F24" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G24" t="s">
         <v>3</v>
@@ -1335,10 +1327,10 @@
         <v>66</v>
       </c>
       <c r="E25" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F25" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G25" t="s">
         <v>3</v>
@@ -1361,10 +1353,10 @@
         <v>64</v>
       </c>
       <c r="E26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F26" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G26" t="s">
         <v>3</v>
@@ -1387,10 +1379,10 @@
         <v>62</v>
       </c>
       <c r="E27" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F27" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G27" t="s">
         <v>3</v>
@@ -1413,10 +1405,10 @@
         <v>62</v>
       </c>
       <c r="E28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F28" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G28" t="s">
         <v>3</v>
@@ -1439,10 +1431,10 @@
         <v>61</v>
       </c>
       <c r="E29" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F29" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G29" t="s">
         <v>3</v>
@@ -1465,10 +1457,10 @@
         <v>62</v>
       </c>
       <c r="E30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F30" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G30" t="s">
         <v>3</v>
@@ -1491,10 +1483,10 @@
         <v>62</v>
       </c>
       <c r="E31" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F31" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G31" t="s">
         <v>3</v>
@@ -1517,10 +1509,10 @@
         <v>66</v>
       </c>
       <c r="E32" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F32" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G32" t="s">
         <v>3</v>
@@ -1543,71 +1535,62 @@
         <v>66</v>
       </c>
       <c r="E33" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F33" t="s">
+        <v>80</v>
+      </c>
+      <c r="G33" t="s">
+        <v>3</v>
+      </c>
+      <c r="H33" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>29</v>
+      </c>
+      <c r="B34" t="s">
         <v>82</v>
       </c>
-      <c r="G33" t="s">
-        <v>3</v>
-      </c>
-      <c r="H33" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="2" t="s">
+      <c r="C34" t="s">
+        <v>35</v>
+      </c>
+      <c r="D34" t="s">
+        <v>66</v>
+      </c>
+      <c r="E34" t="s">
+        <v>76</v>
+      </c>
+      <c r="F34" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A35" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B35" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="D35" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>47</v>
-      </c>
-      <c r="B35" t="s">
-        <v>48</v>
-      </c>
-      <c r="C35" t="s">
-        <v>49</v>
-      </c>
-      <c r="D35" t="s">
-        <v>66</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="G35" t="s">
-        <v>3</v>
-      </c>
-      <c r="H35" t="s">
-        <v>70</v>
-      </c>
-      <c r="I35" t="s">
-        <v>71</v>
+      <c r="E35" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
@@ -1615,7 +1598,7 @@
         <v>47</v>
       </c>
       <c r="B36" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C36" t="s">
         <v>49</v>
@@ -1624,10 +1607,10 @@
         <v>66</v>
       </c>
       <c r="E36" t="s">
-        <v>77</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>82</v>
+        <v>76</v>
+      </c>
+      <c r="F36" t="s">
+        <v>80</v>
       </c>
       <c r="G36" t="s">
         <v>3</v>
@@ -1644,25 +1627,28 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C37" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D37" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E37" t="s">
-        <v>75</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>82</v>
+        <v>76</v>
+      </c>
+      <c r="F37" t="s">
+        <v>80</v>
       </c>
       <c r="G37" t="s">
         <v>3</v>
       </c>
       <c r="H37" t="s">
         <v>70</v>
+      </c>
+      <c r="I37" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
@@ -1670,28 +1656,25 @@
         <v>47</v>
       </c>
       <c r="B38" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C38" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D38" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E38" t="s">
-        <v>77</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>82</v>
+        <v>74</v>
+      </c>
+      <c r="F38" t="s">
+        <v>80</v>
       </c>
       <c r="G38" t="s">
         <v>3</v>
       </c>
       <c r="H38" t="s">
         <v>70</v>
-      </c>
-      <c r="I38" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
@@ -1699,22 +1682,22 @@
         <v>47</v>
       </c>
       <c r="B39" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C39" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D39" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E39" t="s">
         <v>76</v>
       </c>
-      <c r="F39" s="3" t="s">
-        <v>82</v>
+      <c r="F39" t="s">
+        <v>80</v>
       </c>
       <c r="G39" t="s">
-        <v>72</v>
+        <v>3</v>
       </c>
       <c r="H39" t="s">
         <v>70</v>
@@ -1728,7 +1711,7 @@
         <v>47</v>
       </c>
       <c r="B40" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="C40" t="s">
         <v>52</v>
@@ -1737,13 +1720,13 @@
         <v>62</v>
       </c>
       <c r="E40" t="s">
-        <v>76</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>82</v>
+        <v>75</v>
+      </c>
+      <c r="F40" t="s">
+        <v>80</v>
       </c>
       <c r="G40" t="s">
-        <v>72</v>
+        <v>3</v>
       </c>
       <c r="H40" t="s">
         <v>70</v>
@@ -1757,19 +1740,19 @@
         <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C41" t="s">
         <v>52</v>
       </c>
       <c r="D41" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E41" t="s">
-        <v>75</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>82</v>
+        <v>76</v>
+      </c>
+      <c r="F41" t="s">
+        <v>80</v>
       </c>
       <c r="G41" t="s">
         <v>3</v>
@@ -1786,7 +1769,7 @@
         <v>47</v>
       </c>
       <c r="B42" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C42" t="s">
         <v>52</v>
@@ -1795,13 +1778,13 @@
         <v>61</v>
       </c>
       <c r="E42" t="s">
-        <v>75</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>82</v>
+        <v>74</v>
+      </c>
+      <c r="F42" t="s">
+        <v>80</v>
       </c>
       <c r="G42" t="s">
-        <v>72</v>
+        <v>3</v>
       </c>
       <c r="H42" t="s">
         <v>70</v>
@@ -1815,22 +1798,28 @@
         <v>47</v>
       </c>
       <c r="B43" t="s">
-        <v>78</v>
-      </c>
-      <c r="C43" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C43" t="s">
         <v>52</v>
       </c>
       <c r="D43" t="s">
         <v>61</v>
       </c>
       <c r="E43" t="s">
-        <v>75</v>
-      </c>
-      <c r="F43" s="3" t="s">
-        <v>82</v>
+        <v>74</v>
+      </c>
+      <c r="F43" t="s">
+        <v>80</v>
       </c>
       <c r="G43" t="s">
-        <v>81</v>
+        <v>3</v>
+      </c>
+      <c r="H43" t="s">
+        <v>70</v>
+      </c>
+      <c r="I43" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
@@ -1838,19 +1827,48 @@
         <v>47</v>
       </c>
       <c r="B44" t="s">
+        <v>77</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D44" t="s">
+        <v>61</v>
+      </c>
+      <c r="E44" t="s">
+        <v>74</v>
+      </c>
+      <c r="F44" t="s">
+        <v>80</v>
+      </c>
+      <c r="G44" t="s">
+        <v>3</v>
+      </c>
+      <c r="H44" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" t="s">
+        <v>78</v>
+      </c>
+      <c r="C45" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C44" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D44" t="s">
-        <v>77</v>
-      </c>
-      <c r="E44" t="s">
-        <v>77</v>
-      </c>
-      <c r="G44" t="s">
-        <v>81</v>
+      <c r="D45" t="s">
+        <v>76</v>
+      </c>
+      <c r="E45" t="s">
+        <v>76</v>
+      </c>
+      <c r="G45" t="s">
+        <v>3</v>
+      </c>
+      <c r="H45" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>